<commit_message>
Integrate 4.0.4: commit #6dbabe8, 2/3/25, Block all offshore wind not currently planned/under construction in Current Policies
</commit_message>
<xml_diff>
--- a/InputData/elec/BBNPPTY/BAU Ban New Power Plants This Year.xlsx
+++ b/InputData/elec/BBNPPTY/BAU Ban New Power Plants This Year.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\robbie\Models\US\Models\eps-us\InputData\elec\BBNPPTY\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Modeling\EPS\US\eps-us\InputData\elec\BBNPPTY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AED5C7C3-C6DD-4CC0-A75D-D5DA17DC76DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FD9606DE-C9CB-45C7-B0C5-5718740EFEDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3900" yWindow="3900" windowWidth="38865" windowHeight="17235" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
     <t>Source:</t>
   </si>
@@ -141,6 +141,15 @@
   </si>
   <si>
     <t>and the construction time for new or modified plants.</t>
+  </si>
+  <si>
+    <t>Due to recent blocks on offshore wind permitting and leasing, we assume only</t>
+  </si>
+  <si>
+    <t>already planned capacity (captured in elec/BPMCCS) will be built, and other</t>
+  </si>
+  <si>
+    <t>economic or reliability additions will not occur (offshore wind set to 1 in this file).</t>
   </si>
 </sst>
 </file>
@@ -523,18 +532,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B20"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="60.85546875" customWidth="1"/>
+    <col min="2" max="2" width="60.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -542,54 +551,69 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B5" s="3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B6" s="3">
         <v>2024</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B7" s="4" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>2028</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>35</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -604,13 +628,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" customWidth="1"/>
-    <col min="2" max="2" width="27.28515625" customWidth="1"/>
+    <col min="1" max="1" width="26.453125" customWidth="1"/>
+    <col min="2" max="2" width="27.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -705,7 +729,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -800,7 +824,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -895,7 +919,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -990,7 +1014,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -1085,7 +1109,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -1180,7 +1204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -1275,7 +1299,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1370,7 +1394,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -1465,7 +1489,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -1560,7 +1584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -1655,7 +1679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -1750,7 +1774,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -1845,7 +1869,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>10</v>
       </c>
@@ -1940,7 +1964,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -1953,89 +1977,89 @@
       <c r="D15">
         <v>1</v>
       </c>
-      <c r="E15" s="5">
-        <v>0</v>
-      </c>
-      <c r="F15" s="5">
-        <v>0</v>
-      </c>
-      <c r="G15" s="5">
-        <v>0</v>
-      </c>
-      <c r="H15" s="5">
-        <v>0</v>
-      </c>
-      <c r="I15" s="5">
-        <v>0</v>
-      </c>
-      <c r="J15" s="5">
-        <v>0</v>
-      </c>
-      <c r="K15" s="5">
-        <v>0</v>
-      </c>
-      <c r="L15" s="5">
-        <v>0</v>
-      </c>
-      <c r="M15" s="5">
-        <v>0</v>
-      </c>
-      <c r="N15" s="5">
-        <v>0</v>
-      </c>
-      <c r="O15" s="5">
-        <v>0</v>
-      </c>
-      <c r="P15" s="5">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="5">
-        <v>0</v>
-      </c>
-      <c r="R15" s="5">
-        <v>0</v>
-      </c>
-      <c r="S15" s="5">
-        <v>0</v>
-      </c>
-      <c r="T15" s="5">
-        <v>0</v>
-      </c>
-      <c r="U15" s="5">
-        <v>0</v>
-      </c>
-      <c r="V15" s="5">
-        <v>0</v>
-      </c>
-      <c r="W15" s="5">
-        <v>0</v>
-      </c>
-      <c r="X15" s="5">
-        <v>0</v>
-      </c>
-      <c r="Y15" s="5">
-        <v>0</v>
-      </c>
-      <c r="Z15" s="5">
-        <v>0</v>
-      </c>
-      <c r="AA15" s="5">
-        <v>0</v>
-      </c>
-      <c r="AB15" s="5">
-        <v>0</v>
-      </c>
-      <c r="AC15" s="5">
-        <v>0</v>
-      </c>
-      <c r="AD15" s="5">
-        <v>0</v>
-      </c>
-      <c r="AE15" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15">
+        <v>1</v>
+      </c>
+      <c r="H15">
+        <v>1</v>
+      </c>
+      <c r="I15">
+        <v>1</v>
+      </c>
+      <c r="J15">
+        <v>1</v>
+      </c>
+      <c r="K15">
+        <v>1</v>
+      </c>
+      <c r="L15">
+        <v>1</v>
+      </c>
+      <c r="M15">
+        <v>1</v>
+      </c>
+      <c r="N15">
+        <v>1</v>
+      </c>
+      <c r="O15">
+        <v>1</v>
+      </c>
+      <c r="P15">
+        <v>1</v>
+      </c>
+      <c r="Q15">
+        <v>1</v>
+      </c>
+      <c r="R15">
+        <v>1</v>
+      </c>
+      <c r="S15">
+        <v>1</v>
+      </c>
+      <c r="T15">
+        <v>1</v>
+      </c>
+      <c r="U15">
+        <v>1</v>
+      </c>
+      <c r="V15">
+        <v>1</v>
+      </c>
+      <c r="W15">
+        <v>1</v>
+      </c>
+      <c r="X15">
+        <v>1</v>
+      </c>
+      <c r="Y15">
+        <v>1</v>
+      </c>
+      <c r="Z15">
+        <v>1</v>
+      </c>
+      <c r="AA15">
+        <v>1</v>
+      </c>
+      <c r="AB15">
+        <v>1</v>
+      </c>
+      <c r="AC15">
+        <v>1</v>
+      </c>
+      <c r="AD15">
+        <v>1</v>
+      </c>
+      <c r="AE15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -2130,7 +2154,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -2225,7 +2249,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -2320,7 +2344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>20</v>
       </c>
@@ -2415,7 +2439,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -2510,7 +2534,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>22</v>
       </c>
@@ -2605,7 +2629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -2700,7 +2724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>24</v>
       </c>
@@ -2795,7 +2819,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A24" s="6" t="s">
         <v>25</v>
       </c>
@@ -2890,7 +2914,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A25" s="6" t="s">
         <v>26</v>
       </c>

</xml_diff>

<commit_message>
Integrate 4.0.4, commit #68484fb, 2/11/25, Update historical capacity additions; for BPMCCS, increase wind and solar additions to cover all capacity currently under construction (other files already integrated via main merge)
</commit_message>
<xml_diff>
--- a/InputData/elec/BBNPPTY/BAU Ban New Power Plants This Year.xlsx
+++ b/InputData/elec/BBNPPTY/BAU Ban New Power Plants This Year.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Modeling\EPS\US\eps-us\InputData\elec\BBNPPTY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FD9606DE-C9CB-45C7-B0C5-5718740EFEDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D074A985-6CC5-4AEA-AF92-B01A9D3FF736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="62850" yWindow="1380" windowWidth="21600" windowHeight="12525" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -743,7 +743,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F2" s="5">
         <v>0</v>
@@ -838,7 +838,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" s="5">
         <v>0</v>
@@ -933,7 +933,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" s="5">
         <v>0</v>
@@ -1028,7 +1028,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" s="5">
         <v>0</v>
@@ -1123,7 +1123,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6" s="5">
         <v>0</v>
@@ -1218,7 +1218,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F7" s="5">
         <v>0</v>
@@ -1313,7 +1313,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" s="5">
         <v>0</v>
@@ -1408,7 +1408,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" s="5">
         <v>0</v>
@@ -1503,7 +1503,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10" s="5">
         <v>0</v>
@@ -1598,7 +1598,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" s="5">
         <v>0</v>
@@ -1693,7 +1693,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12" s="5">
         <v>0</v>
@@ -1788,7 +1788,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" s="5">
         <v>0</v>
@@ -1883,7 +1883,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" s="5">
         <v>0</v>
@@ -1977,7 +1977,7 @@
       <c r="D15">
         <v>1</v>
       </c>
-      <c r="E15">
+      <c r="E15" s="5">
         <v>1</v>
       </c>
       <c r="F15">
@@ -2073,7 +2073,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" s="5">
         <v>0</v>
@@ -2168,7 +2168,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" s="5">
         <v>0</v>
@@ -2263,7 +2263,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F18" s="5">
         <v>0</v>
@@ -2738,7 +2738,7 @@
         <v>1</v>
       </c>
       <c r="E23" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F23" s="5">
         <v>0</v>
@@ -2833,7 +2833,7 @@
         <v>1</v>
       </c>
       <c r="E24" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F24" s="5">
         <v>0</v>
@@ -2928,7 +2928,7 @@
         <v>1</v>
       </c>
       <c r="E25" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25" s="5">
         <v>0</v>

</xml_diff>

<commit_message>
Remove bans for new coal (from 111 rules), ban hydrogen technologies before 2028
</commit_message>
<xml_diff>
--- a/InputData/elec/BBNPPTY/BAU Ban New Power Plants This Year.xlsx
+++ b/InputData/elec/BBNPPTY/BAU Ban New Power Plants This Year.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\BBNPPTY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B5267E0-EC49-461E-990C-D3E82BA1BFF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{385F7B4F-2A1E-47AD-ABA4-C02D7972106A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>Source:</t>
   </si>
@@ -134,12 +134,6 @@
     <t>This is a Boolean value that should be set to 0 or 1 in each year.</t>
   </si>
   <si>
-    <t>In the U.S., we use this to represent EPA 111 Rules. New coal without CCS is banned starting in</t>
-  </si>
-  <si>
-    <t>We also assume no new coal with CCS can be built prior to 2028 given the state of the technology</t>
-  </si>
-  <si>
     <t>and the construction time for new or modified plants.</t>
   </si>
   <si>
@@ -165,6 +159,9 @@
   </si>
   <si>
     <t>(planned additions according to EIA are included in elec/BPMCCS)</t>
+  </si>
+  <si>
+    <t>We also assume no new coal with CCS or hydrogen can be built prior to 2028 given the state of the technology</t>
   </si>
 </sst>
 </file>
@@ -547,18 +544,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B27"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B24"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="60.85546875" customWidth="1"/>
+    <col min="2" max="2" width="60.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -566,94 +563,84 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B5" s="3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B6" s="3">
         <v>2024</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B7" s="4" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>2028</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
         <v>41</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -668,13 +655,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" customWidth="1"/>
-    <col min="2" max="2" width="27.28515625" customWidth="1"/>
+    <col min="1" max="1" width="26.453125" customWidth="1"/>
+    <col min="2" max="2" width="27.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -769,7 +756,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -795,76 +782,76 @@
         <v>0</v>
       </c>
       <c r="I2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD2" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE2" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -959,7 +946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -1054,7 +1041,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -1149,7 +1136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -1244,7 +1231,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -1339,7 +1326,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1434,7 +1421,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -1529,7 +1516,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -1624,7 +1611,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -1719,7 +1706,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -1814,7 +1801,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -1909,7 +1896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>10</v>
       </c>
@@ -1935,76 +1922,76 @@
         <v>0</v>
       </c>
       <c r="I14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD14" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE14" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -2099,7 +2086,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -2194,7 +2181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -2289,7 +2276,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -2384,7 +2371,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>20</v>
       </c>
@@ -2479,7 +2466,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -2574,7 +2561,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>22</v>
       </c>
@@ -2669,7 +2656,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -2764,7 +2751,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>24</v>
       </c>
@@ -2781,13 +2768,13 @@
         <v>1</v>
       </c>
       <c r="F23" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G23" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H23" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I23" s="5">
         <v>0</v>
@@ -2859,7 +2846,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A24" s="6" t="s">
         <v>25</v>
       </c>
@@ -2876,13 +2863,13 @@
         <v>1</v>
       </c>
       <c r="F24" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H24" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I24" s="5">
         <v>0</v>
@@ -2954,7 +2941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A25" s="6" t="s">
         <v>26</v>
       </c>
@@ -2971,13 +2958,13 @@
         <v>1</v>
       </c>
       <c r="F25" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H25" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I25" s="5">
         <v>0</v>

</xml_diff>

<commit_message>
Disallow non-mandated onshore wind in 2026 for permitting reasons
</commit_message>
<xml_diff>
--- a/InputData/elec/BBNPPTY/BAU Ban New Power Plants This Year.xlsx
+++ b/InputData/elec/BBNPPTY/BAU Ban New Power Plants This Year.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\BBNPPTY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0EFE6CE-B1E1-414D-B79D-B8405EC59DD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04181323-3746-4842-866D-0CBCE32CC42C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>Source:</t>
   </si>
@@ -153,6 +153,15 @@
   </si>
   <si>
     <t>that these plants have a 6 year lead time and therefore cannot be built for economic reasons before 2032</t>
+  </si>
+  <si>
+    <t xml:space="preserve">We disallow new onshore wind (other than policy mandated capacity) in 2026 under </t>
+  </si>
+  <si>
+    <t>the assumption that any new wind not already in progress would not receive permits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">on time. </t>
   </si>
 </sst>
 </file>
@@ -521,7 +530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="60.81640625" customWidth="1"/>
@@ -598,6 +607,21 @@
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>35</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -1144,7 +1168,7 @@
         <v>1</v>
       </c>
       <c r="D7" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" s="3">
         <v>0</v>

</xml_diff>

<commit_message>
Ban new CCUS plants, SMR, H2 pre-2031
</commit_message>
<xml_diff>
--- a/InputData/elec/BBNPPTY/BAU Ban New Power Plants This Year.xlsx
+++ b/InputData/elec/BBNPPTY/BAU Ban New Power Plants This Year.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\BBNPPTY\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\elec\BBNPPTY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04181323-3746-4842-866D-0CBCE32CC42C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DAB78AC-FAE4-440F-985C-291D7E28BAA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-27285" yWindow="1515" windowWidth="22290" windowHeight="13995" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -143,9 +143,6 @@
     <t>(planned additions according to EIA are included in elec/BPMCCS)</t>
   </si>
   <si>
-    <t>We also assume no new coal with CCS or hydrogen can be built prior to 2028 given the state of the technology</t>
-  </si>
-  <si>
     <t>For historical years, we directly read in capacity additions in other input</t>
   </si>
   <si>
@@ -162,6 +159,9 @@
   </si>
   <si>
     <t xml:space="preserve">on time. </t>
+  </si>
+  <si>
+    <t>We also assume no new coal with CCS or hydrogen can be built prior to 2030 given the state of the technology</t>
   </si>
 </sst>
 </file>
@@ -531,97 +531,97 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B24"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="60.81640625" customWidth="1"/>
+    <col min="2" max="2" width="60.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>41</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -636,12 +636,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AB25"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.453125" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -727,7 +727,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -813,7 +813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -899,7 +899,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -985,7 +985,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -1071,7 +1071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -1157,7 +1157,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -1243,7 +1243,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1329,7 +1329,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -1415,7 +1415,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -1501,7 +1501,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -1587,7 +1587,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -1673,7 +1673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -1759,7 +1759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>10</v>
       </c>
@@ -1845,7 +1845,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -1931,7 +1931,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -2017,7 +2017,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -2103,7 +2103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -2189,7 +2189,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>20</v>
       </c>
@@ -2202,17 +2202,17 @@
       <c r="D19" s="3">
         <v>1</v>
       </c>
-      <c r="E19" s="3">
-        <v>1</v>
-      </c>
-      <c r="F19" s="3">
-        <v>0</v>
-      </c>
-      <c r="G19" s="3">
-        <v>0</v>
-      </c>
-      <c r="H19" s="3">
-        <v>0</v>
+      <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="F19">
+        <v>1</v>
+      </c>
+      <c r="G19">
+        <v>1</v>
+      </c>
+      <c r="H19">
+        <v>1</v>
       </c>
       <c r="I19" s="3">
         <v>0</v>
@@ -2275,7 +2275,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -2288,17 +2288,17 @@
       <c r="D20" s="3">
         <v>1</v>
       </c>
-      <c r="E20" s="3">
-        <v>1</v>
-      </c>
-      <c r="F20" s="3">
-        <v>0</v>
-      </c>
-      <c r="G20" s="3">
-        <v>0</v>
-      </c>
-      <c r="H20" s="3">
-        <v>0</v>
+      <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="F20">
+        <v>1</v>
+      </c>
+      <c r="G20">
+        <v>1</v>
+      </c>
+      <c r="H20">
+        <v>1</v>
       </c>
       <c r="I20" s="3">
         <v>0</v>
@@ -2361,7 +2361,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>22</v>
       </c>
@@ -2374,17 +2374,17 @@
       <c r="D21" s="3">
         <v>1</v>
       </c>
-      <c r="E21" s="3">
-        <v>1</v>
-      </c>
-      <c r="F21" s="3">
-        <v>0</v>
-      </c>
-      <c r="G21" s="3">
-        <v>0</v>
-      </c>
-      <c r="H21" s="3">
-        <v>0</v>
+      <c r="E21">
+        <v>1</v>
+      </c>
+      <c r="F21">
+        <v>1</v>
+      </c>
+      <c r="G21">
+        <v>1</v>
+      </c>
+      <c r="H21">
+        <v>1</v>
       </c>
       <c r="I21" s="3">
         <v>0</v>
@@ -2447,7 +2447,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -2460,17 +2460,17 @@
       <c r="D22" s="3">
         <v>1</v>
       </c>
-      <c r="E22" s="3">
-        <v>1</v>
-      </c>
-      <c r="F22" s="3">
-        <v>0</v>
-      </c>
-      <c r="G22" s="3">
-        <v>0</v>
-      </c>
-      <c r="H22" s="3">
-        <v>0</v>
+      <c r="E22">
+        <v>1</v>
+      </c>
+      <c r="F22">
+        <v>1</v>
+      </c>
+      <c r="G22">
+        <v>1</v>
+      </c>
+      <c r="H22">
+        <v>1</v>
       </c>
       <c r="I22" s="3">
         <v>0</v>
@@ -2533,7 +2533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>24</v>
       </c>
@@ -2546,17 +2546,17 @@
       <c r="D23" s="3">
         <v>1</v>
       </c>
-      <c r="E23" s="3">
-        <v>1</v>
-      </c>
-      <c r="F23" s="3">
-        <v>0</v>
-      </c>
-      <c r="G23" s="3">
-        <v>0</v>
-      </c>
-      <c r="H23" s="3">
-        <v>0</v>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
+        <v>1</v>
+      </c>
+      <c r="G23">
+        <v>1</v>
+      </c>
+      <c r="H23">
+        <v>1</v>
       </c>
       <c r="I23" s="3">
         <v>0</v>
@@ -2619,7 +2619,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
         <v>25</v>
       </c>
@@ -2632,17 +2632,17 @@
       <c r="D24" s="3">
         <v>1</v>
       </c>
-      <c r="E24" s="3">
-        <v>1</v>
-      </c>
-      <c r="F24" s="3">
-        <v>0</v>
-      </c>
-      <c r="G24" s="3">
-        <v>0</v>
-      </c>
-      <c r="H24" s="3">
-        <v>0</v>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24">
+        <v>1</v>
+      </c>
+      <c r="G24">
+        <v>1</v>
+      </c>
+      <c r="H24">
+        <v>1</v>
       </c>
       <c r="I24" s="3">
         <v>0</v>
@@ -2705,7 +2705,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
         <v>26</v>
       </c>
@@ -2718,17 +2718,17 @@
       <c r="D25" s="3">
         <v>1</v>
       </c>
-      <c r="E25" s="3">
-        <v>1</v>
-      </c>
-      <c r="F25" s="3">
-        <v>0</v>
-      </c>
-      <c r="G25" s="3">
-        <v>0</v>
-      </c>
-      <c r="H25" s="3">
-        <v>0</v>
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="F25">
+        <v>1</v>
+      </c>
+      <c r="G25">
+        <v>1</v>
+      </c>
+      <c r="H25">
+        <v>1</v>
       </c>
       <c r="I25" s="3">
         <v>0</v>

</xml_diff>

<commit_message>
Adds hard/soft cap on elec builds; calibrates future years
</commit_message>
<xml_diff>
--- a/InputData/elec/BBNPPTY/BAU Ban New Power Plants This Year.xlsx
+++ b/InputData/elec/BBNPPTY/BAU Ban New Power Plants This Year.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\elec\BBNPPTY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DAB78AC-FAE4-440F-985C-291D7E28BAA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AE63472-43E3-4596-94E0-7B5A9AEBD943}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27285" yWindow="1515" windowWidth="22290" windowHeight="13995" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="380" yWindow="380" windowWidth="17220" windowHeight="10710" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -131,9 +131,6 @@
     <t>already planned capacity (captured in elec/BPMCCS) will be built, and other</t>
   </si>
   <si>
-    <t>economic or reliability additions will not occur (offshore wind set to 1 in this file).</t>
-  </si>
-  <si>
     <t>data files and therefore disallow additional economic additions.</t>
   </si>
   <si>
@@ -162,6 +159,9 @@
   </si>
   <si>
     <t>We also assume no new coal with CCS or hydrogen can be built prior to 2030 given the state of the technology</t>
+  </si>
+  <si>
+    <t>economic or reliability additions will not occur until 2032.</t>
   </si>
 </sst>
 </file>
@@ -531,97 +531,97 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B24"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="60.85546875" customWidth="1"/>
+    <col min="2" max="2" width="60.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
         <v>40</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -636,12 +636,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AB25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" customWidth="1"/>
+    <col min="1" max="1" width="26.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -727,7 +727,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -813,7 +813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -899,7 +899,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -985,7 +985,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -1071,7 +1071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -1157,7 +1157,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -1243,7 +1243,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1329,7 +1329,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -1415,7 +1415,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -1501,7 +1501,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -1587,7 +1587,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -1673,7 +1673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -1759,7 +1759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>10</v>
       </c>
@@ -1845,7 +1845,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -1871,67 +1871,67 @@
         <v>1</v>
       </c>
       <c r="I15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -2017,7 +2017,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -2103,7 +2103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -2189,7 +2189,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>20</v>
       </c>
@@ -2275,7 +2275,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -2361,7 +2361,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>22</v>
       </c>
@@ -2447,7 +2447,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -2533,7 +2533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>24</v>
       </c>
@@ -2619,7 +2619,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A24" s="4" t="s">
         <v>25</v>
       </c>
@@ -2705,7 +2705,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A25" s="4" t="s">
         <v>26</v>
       </c>

</xml_diff>

<commit_message>
ban geothermal until 2031 BBNPPTY
</commit_message>
<xml_diff>
--- a/InputData/elec/BBNPPTY/BAU Ban New Power Plants This Year.xlsx
+++ b/InputData/elec/BBNPPTY/BAU Ban New Power Plants This Year.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\elec\BBNPPTY\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OliviaAshmoore\Documents\Github Repos\eps-us\InputData\elec\BBNPPTY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AE63472-43E3-4596-94E0-7B5A9AEBD943}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7487E94-2E26-4C24-B6A2-CA909A2A2301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="380" windowWidth="17220" windowHeight="10710" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6855" yWindow="270" windowWidth="21600" windowHeight="12405" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -531,17 +531,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B24"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="60.81640625" customWidth="1"/>
+    <col min="2" max="2" width="60.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -549,77 +549,77 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>40</v>
       </c>
@@ -636,12 +636,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AB25"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.453125" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -727,7 +727,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -813,7 +813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -899,7 +899,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -985,7 +985,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -1071,7 +1071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -1157,7 +1157,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -1243,7 +1243,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1329,7 +1329,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -1415,7 +1415,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -1501,7 +1501,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -1511,20 +1511,20 @@
       <c r="C11">
         <v>1</v>
       </c>
-      <c r="D11" s="3">
-        <v>0</v>
-      </c>
-      <c r="E11" s="3">
-        <v>0</v>
-      </c>
-      <c r="F11" s="3">
-        <v>0</v>
-      </c>
-      <c r="G11" s="3">
-        <v>0</v>
-      </c>
-      <c r="H11" s="3">
-        <v>0</v>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
+        <v>1</v>
       </c>
       <c r="I11" s="3">
         <v>0</v>
@@ -1587,7 +1587,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -1673,7 +1673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -1759,7 +1759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>10</v>
       </c>
@@ -1845,7 +1845,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -1931,7 +1931,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -2017,7 +2017,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -2103,7 +2103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -2189,7 +2189,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>20</v>
       </c>
@@ -2275,7 +2275,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -2361,7 +2361,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>22</v>
       </c>
@@ -2447,7 +2447,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -2533,7 +2533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>24</v>
       </c>
@@ -2619,7 +2619,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
         <v>25</v>
       </c>
@@ -2705,7 +2705,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
         <v>26</v>
       </c>

</xml_diff>